<commit_message>
Scaling non geo-features, k=35
</commit_message>
<xml_diff>
--- a/results/CA/final_results.xlsx
+++ b/results/CA/final_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\mamintoosi-papers-codes\House2Vec\results\CA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05AEE9D9-4302-4E5F-9F6A-896685E0BA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965DACD2-FD43-4262-82C6-DF88B82F04C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7185" yWindow="1440" windowWidth="11565" windowHeight="11340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Model</t>
   </si>
@@ -38,24 +38,6 @@
   </si>
   <si>
     <t>MSE_log</t>
-  </si>
-  <si>
-    <t>GradientBoosting (Raw)</t>
-  </si>
-  <si>
-    <t>RandomForest (Raw)</t>
-  </si>
-  <si>
-    <t>GradientBoosting (DeepWalk-ed2-nw50-wl15)</t>
-  </si>
-  <si>
-    <t>RandomForest (DeepWalk-ed2-nw50-wl15)</t>
-  </si>
-  <si>
-    <t>GradientBoosting (Node2Vec-ed2-nw50-wl15-p1-q1)</t>
-  </si>
-  <si>
-    <t>RandomForest (Node2Vec-ed2-nw50-wl15-p1-q1)</t>
   </si>
   <si>
     <t>GradientBoosting (Node2Vec-ed2-nw50-wl15-p3-q1)</t>
@@ -424,10 +406,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.140625" customWidth="1"/>
+    <col min="1" max="1" width="55" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -455,19 +437,19 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>0.7867993259399797</v>
+        <v>0.7854999239250825</v>
       </c>
       <c r="C2">
-        <v>0.2107531635705186</v>
+        <v>0.21030523803828649</v>
       </c>
       <c r="D2">
-        <v>0.60665362035225046</v>
+        <v>0.60812133072407049</v>
       </c>
       <c r="E2">
-        <v>54214.652720339247</v>
+        <v>54379.613775771271</v>
       </c>
       <c r="F2">
-        <v>1.302204289605996E-2</v>
+        <v>1.302255285530386E-2</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -475,139 +457,19 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>0.83843904749276565</v>
+        <v>0.83445519763897402</v>
       </c>
       <c r="C3">
-        <v>0.16590272194865141</v>
+        <v>0.16951007456562581</v>
       </c>
       <c r="D3">
-        <v>0.72749510763209391</v>
+        <v>0.71917808219178081</v>
       </c>
       <c r="E3">
-        <v>47194.413782685428</v>
+        <v>47772.741914136866</v>
       </c>
       <c r="F3">
-        <v>9.3672504138372324E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4">
-        <v>0.78218035402301045</v>
-      </c>
-      <c r="C4">
-        <v>0.21296300460085471</v>
-      </c>
-      <c r="D4">
-        <v>0.6071428571428571</v>
-      </c>
-      <c r="E4">
-        <v>54798.783484290587</v>
-      </c>
-      <c r="F4">
-        <v>1.335453609746517E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>0.83293428285652948</v>
-      </c>
-      <c r="C5">
-        <v>0.16951150901822201</v>
-      </c>
-      <c r="D5">
-        <v>0.72455968688845396</v>
-      </c>
-      <c r="E5">
-        <v>47991.692152065603</v>
-      </c>
-      <c r="F5">
-        <v>9.6853853212935034E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6">
-        <v>0.78411631561318706</v>
-      </c>
-      <c r="C6">
-        <v>0.2088098354234362</v>
-      </c>
-      <c r="D6">
-        <v>0.6154598825831703</v>
-      </c>
-      <c r="E6">
-        <v>54554.716612189448</v>
-      </c>
-      <c r="F6">
-        <v>1.2934473098799269E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7">
-        <v>0.83509625898697581</v>
-      </c>
-      <c r="C7">
-        <v>0.1697697589200228</v>
-      </c>
-      <c r="D7">
-        <v>0.71575342465753422</v>
-      </c>
-      <c r="E7">
-        <v>47680.15379294083</v>
-      </c>
-      <c r="F7">
-        <v>9.7072895770188745E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8">
-        <v>0.78825611839847121</v>
-      </c>
-      <c r="C8">
-        <v>0.20785606000108581</v>
-      </c>
-      <c r="D8">
-        <v>0.61154598825831707</v>
-      </c>
-      <c r="E8">
-        <v>54029.111852571812</v>
-      </c>
-      <c r="F8">
-        <v>1.284654527467052E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9">
-        <v>0.8360665261511443</v>
-      </c>
-      <c r="C9">
-        <v>0.16805564703961251</v>
-      </c>
-      <c r="D9">
-        <v>0.72064579256360073</v>
-      </c>
-      <c r="E9">
-        <v>47539.675661501293</v>
-      </c>
-      <c r="F9">
-        <v>9.4106003601255508E-3</v>
+        <v>9.6647739953038009E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
k=10 is also bad
</commit_message>
<xml_diff>
--- a/results/CA/final_results.xlsx
+++ b/results/CA/final_results.xlsx
@@ -1,72 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\mamintoosi-papers-codes\House2Vec\results\CA\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965DACD2-FD43-4262-82C6-DF88B82F04C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="7185" yWindow="1440" windowWidth="11565" windowHeight="11340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Model</t>
-  </si>
-  <si>
-    <t>R2</t>
-  </si>
-  <si>
-    <t>MAPE</t>
-  </si>
-  <si>
-    <t>Accuracy</t>
-  </si>
-  <si>
-    <t>RMSE</t>
-  </si>
-  <si>
-    <t>MSE_log</t>
-  </si>
-  <si>
-    <t>GradientBoosting (Node2Vec-ed2-nw50-wl15-p3-q1)</t>
-  </si>
-  <si>
-    <t>RandomForest (Node2Vec-ed2-nw50-wl15-p3-q1)</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -81,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -405,71 +420,88 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="55" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MAPE</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MSE_log</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>0.7854999239250825</v>
-      </c>
-      <c r="C2">
-        <v>0.21030523803828649</v>
-      </c>
-      <c r="D2">
-        <v>0.60812133072407049</v>
-      </c>
-      <c r="E2">
-        <v>54379.613775771271</v>
-      </c>
-      <c r="F2">
-        <v>1.302255285530386E-2</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GradientBoosting (Node2Vec-ed2-nw50-wl15-p3-q1)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.7873316349518172</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.2096980250296688</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.6105675146771037</v>
+      </c>
+      <c r="E2" t="n">
+        <v>54146.93017614674</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.01303012635954701</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>0.83445519763897402</v>
-      </c>
-      <c r="C3">
-        <v>0.16951007456562581</v>
-      </c>
-      <c r="D3">
-        <v>0.71917808219178081</v>
-      </c>
-      <c r="E3">
-        <v>47772.741914136866</v>
-      </c>
-      <c r="F3">
-        <v>9.6647739953038009E-3</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RandomForest (Node2Vec-ed2-nw50-wl15-p3-q1)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.8336470601161611</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1708908154881551</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.7186888454011742</v>
+      </c>
+      <c r="E3" t="n">
+        <v>47889.20568309895</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.009800401460937178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>